<commit_message>
added a protein only model
</commit_message>
<xml_diff>
--- a/results/prosmith_results.xlsx
+++ b/results/prosmith_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantmcconachie/Desktop/research/molfeat/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF115A4-A0E7-EF4A-9106-3CACF20FC743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FBF2BB7-EE12-AD4B-ABC8-C231FABA8C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35240" yWindow="-6500" windowWidth="30240" windowHeight="17680" xr2:uid="{123CDDCE-1309-DC46-93B4-EF344A70005B}"/>
+    <workbookView xWindow="-35980" yWindow="-6200" windowWidth="30240" windowHeight="17640" xr2:uid="{123CDDCE-1309-DC46-93B4-EF344A70005B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3290,6 +3290,190 @@
     </row>
   </sheetData>
   <mergeCells count="208">
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="M25:M26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="K21:K22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="M13:M14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L5:L6"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -3314,190 +3498,6 @@
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="K3:K4"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="M13:M14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="M15:M16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="M25:M26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="K27:K28"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="K29:K30"/>
-    <mergeCell ref="L29:L30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>